<commit_message>
Final one-shot scientific reconciliation and release package for ETCCDI Chiang Mai project
Co-authored-by: surasit3173 <247266065+surasit3173@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ETCCDI_ChiangMai/output/statistics/AUTOCORRELATION.xlsx
+++ b/ETCCDI_ChiangMai/output/statistics/AUTOCORRELATION.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,25 +489,35 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>LjungBox_Q5</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>LjungBox_P5</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>LjungBox_P</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Lag1_5_exceed</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>LjungBox_reject</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Serial_dependence_flag</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Primary_method</t>
         </is>
@@ -559,18 +569,24 @@
         <v>0.2552</v>
       </c>
       <c r="O2" t="n">
+        <v>1.289</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.9360619999999999</v>
       </c>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
+      <c r="Q2" t="n">
+        <v>0.9360619999999999</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -622,18 +638,24 @@
         <v>0.2552</v>
       </c>
       <c r="O3" t="n">
+        <v>9.012600000000001</v>
+      </c>
+      <c r="P3" t="n">
         <v>0.108564</v>
       </c>
-      <c r="P3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>0</v>
+      <c r="Q3" t="n">
+        <v>0.108564</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" t="b">
+        <v>0</v>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -685,18 +707,24 @@
         <v>0.2552</v>
       </c>
       <c r="O4" t="n">
+        <v>6.1266</v>
+      </c>
+      <c r="P4" t="n">
         <v>0.294098</v>
       </c>
-      <c r="P4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
+      <c r="Q4" t="n">
+        <v>0.294098</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -748,18 +776,24 @@
         <v>0.2552</v>
       </c>
       <c r="O5" t="n">
+        <v>3.5417</v>
+      </c>
+      <c r="P5" t="n">
         <v>0.6170870000000001</v>
       </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="b">
-        <v>0</v>
+      <c r="Q5" t="n">
+        <v>0.6170870000000001</v>
       </c>
       <c r="R5" t="b">
         <v>0</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -811,18 +845,24 @@
         <v>0.2552</v>
       </c>
       <c r="O6" t="n">
+        <v>7.5049</v>
+      </c>
+      <c r="P6" t="n">
         <v>0.185715</v>
       </c>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="b">
-        <v>0</v>
+      <c r="Q6" t="n">
+        <v>0.185715</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -874,18 +914,24 @@
         <v>0.2552</v>
       </c>
       <c r="O7" t="n">
+        <v>2.9625</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.705772</v>
       </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="b">
-        <v>0</v>
+      <c r="Q7" t="n">
+        <v>0.705772</v>
       </c>
       <c r="R7" t="b">
         <v>0</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S7" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -937,18 +983,24 @@
         <v>0.2552</v>
       </c>
       <c r="O8" t="n">
+        <v>4.2807</v>
+      </c>
+      <c r="P8" t="n">
         <v>0.509753</v>
       </c>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="b">
-        <v>0</v>
+      <c r="Q8" t="n">
+        <v>0.509753</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S8" t="b">
+        <v>0</v>
+      </c>
+      <c r="T8" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -1000,18 +1052,24 @@
         <v>0.2552</v>
       </c>
       <c r="O9" t="n">
+        <v>0.9394</v>
+      </c>
+      <c r="P9" t="n">
         <v>0.967305</v>
       </c>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="b">
-        <v>0</v>
+      <c r="Q9" t="n">
+        <v>0.967305</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S9" t="b">
+        <v>0</v>
+      </c>
+      <c r="T9" t="b">
+        <v>0</v>
+      </c>
+      <c r="U9" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -1063,18 +1121,24 @@
         <v>0.2552</v>
       </c>
       <c r="O10" t="n">
+        <v>10.6865</v>
+      </c>
+      <c r="P10" t="n">
         <v>0.057962</v>
       </c>
-      <c r="P10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q10" t="b">
-        <v>0</v>
+      <c r="Q10" t="n">
+        <v>0.057962</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S10" t="b">
+        <v>0</v>
+      </c>
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>Hamed_Rao_modified_MK</t>
         </is>
@@ -1126,18 +1190,24 @@
         <v>0.2552</v>
       </c>
       <c r="O11" t="n">
+        <v>6.8291</v>
+      </c>
+      <c r="P11" t="n">
         <v>0.233668</v>
       </c>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="b">
-        <v>0</v>
+      <c r="Q11" t="n">
+        <v>0.233668</v>
       </c>
       <c r="R11" t="b">
         <v>0</v>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S11" t="b">
+        <v>0</v>
+      </c>
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" t="inlineStr">
         <is>
           <t>Ordinary_MK</t>
         </is>
@@ -1189,18 +1259,24 @@
         <v>0.2552</v>
       </c>
       <c r="O12" t="n">
+        <v>6.1959</v>
+      </c>
+      <c r="P12" t="n">
         <v>0.287624</v>
       </c>
-      <c r="P12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="b">
-        <v>0</v>
+      <c r="Q12" t="n">
+        <v>0.287624</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S12" t="b">
+        <v>0</v>
+      </c>
+      <c r="T12" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12" t="inlineStr">
         <is>
           <t>Hamed_Rao_modified_MK</t>
         </is>

</xml_diff>